<commit_message>
The knapsack feature has a bug.
</commit_message>
<xml_diff>
--- a/Assets/ArtRes/Excel/道具配置表.xlsx
+++ b/Assets/ArtRes/Excel/道具配置表.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="25600" windowHeight="10480"/>
+    <workbookView windowWidth="13070" windowHeight="4410"/>
   </bookViews>
   <sheets>
     <sheet name="PropInfo" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
+  <si>
+    <t>id</t>
+  </si>
   <si>
     <t>名字</t>
   </si>
@@ -45,6 +48,9 @@
   </si>
   <si>
     <t>maxValue</t>
+  </si>
+  <si>
+    <t>int</t>
   </si>
   <si>
     <t>string</t>
@@ -1012,15 +1018,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="2"/>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelCol="3"/>
   <cols>
-    <col min="1" max="1" width="19.0909090909091" customWidth="1"/>
-    <col min="2" max="2" width="11.8181818181818" customWidth="1"/>
-    <col min="3" max="3" width="20.8181818181818" customWidth="1"/>
+    <col min="1" max="1" width="7.36363636363636" customWidth="1"/>
+    <col min="2" max="2" width="15.3636363636364" customWidth="1"/>
+    <col min="3" max="3" width="13.6363636363636" customWidth="1"/>
+    <col min="4" max="4" width="21.1818181818182" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1030,10 +1037,13 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -1041,97 +1051,124 @@
       <c r="C2" t="s">
         <v>5</v>
       </c>
+      <c r="D2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>0.5</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6">
+        <v>20</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+      <c r="D8">
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>0.5</v>
-      </c>
-      <c r="C5">
+    <row r="9" spans="1:4">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6">
-        <v>20</v>
-      </c>
-      <c r="C6">
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8">
-        <v>1</v>
-      </c>
-      <c r="C8">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-      <c r="C11">
+      <c r="D11">
         <v>0</v>
       </c>
     </row>

</xml_diff>